<commit_message>
Switch dashboard interface to English
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ZDMVQyshdNccdbDjNw8vq
</commit_message>
<xml_diff>
--- a/automation/OPS_Dashboard_Data.xlsx
+++ b/automation/OPS_Dashboard_Data.xlsx
@@ -5592,7 +5592,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Trưởng DX to work with Biên</t>
+          <t>DX lead to work with Biên</t>
         </is>
       </c>
     </row>
@@ -7556,7 +7556,7 @@
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -7613,7 +7613,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cục Tần số</t>
+          <t>Radio Frequency Authority (ARFM)</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cục Tần số</t>
+          <t>Radio Frequency Authority (ARFM)</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -7687,7 +7687,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cục Tần số</t>
+          <t>Radio Frequency Authority (ARFM)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -7724,7 +7724,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cục Tần số</t>
+          <t>Radio Frequency Authority (ARFM)</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cục Tần số</t>
+          <t>Radio Frequency Authority (ARFM)</t>
         </is>
       </c>
       <c r="D6" s="5" t="n"/>
@@ -7782,7 +7782,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cục Tần số</t>
+          <t>Radio Frequency Authority (ARFM)</t>
         </is>
       </c>
       <c r="D7" s="5" t="n"/>
@@ -10736,7 +10736,7 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10769,7 +10769,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Phòng OPS</t>
+          <t>OPS Department</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel dashboard: narrower CBTA chart, value axes at the bottom of bar charts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ZDMVQyshdNccdbDjNw8vq
</commit_message>
<xml_diff>
--- a/automation/OPS_Dashboard_Data.xlsx
+++ b/automation/OPS_Dashboard_Data.xlsx
@@ -899,6 +899,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <legend>
@@ -1016,6 +1017,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <legend>
@@ -1166,6 +1168,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <legend>
@@ -1235,7 +1238,7 @@
       <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6120000" cy="2880000"/>
+    <ext cx="5040000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>

</xml_diff>

<commit_message>
Add PetroVietnam PQPOC logo to web header and Excel Overview
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ZDMVQyshdNccdbDjNw8vq
</commit_message>
<xml_diff>
--- a/automation/OPS_Dashboard_Data.xlsx
+++ b/automation/OPS_Dashboard_Data.xlsx
@@ -1226,6 +1226,31 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>23</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="704850" cy="590550"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 

</xml_diff>

<commit_message>
Archive each report date and add a report picker to view past reports
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ZDMVQyshdNccdbDjNw8vq
</commit_message>
<xml_diff>
--- a/automation/OPS_Dashboard_Data.xlsx
+++ b/automation/OPS_Dashboard_Data.xlsx
@@ -40728,7 +40728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -40783,83 +40783,75 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>5. Power Automate đọc file này theo lịch và đẩy lên dashboard. Sau khi lưu, chờ tới lượt chạy kế tiếp (hoặc chạy tay luồng) rồi 1–2 phút để Vercel cập nhật.</t>
+          <t>5. MỖI KỲ BÁO CÁO: (a) sheet "Thong tin" → sửa report_date thành ngày báo cáo mới; (b) nhập số vào các bảng; (c) xem lại sheet Overview; (d) bấm nút / chạy script "Day so lieu len dashboard". Trang web cập nhật sau 1–2 phút.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Mỗi report_date được lưu thành một bản báo cáo riêng, xem lại trên web ở ô "Report". Đẩy lại cùng report_date sẽ ghi đè bản của ngày đó (dùng để sửa số).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>6. Các sheet dashboard (Overview … Commissioning) ở đầu file tự tính lại ngay khi sửa số; không cần sửa gì trên các sheet đó.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Bảng</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Hiển thị ở</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Cột</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Ý nghĩa</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>meta</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Thong tin</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Ngày báo cáo và tiêu đề (1 dòng duy nhất)</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>report_date</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Ngày báo cáo, dạng YYYY-MM-DD</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>report_title</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Tên báo cáo</t>
         </is>
       </c>
     </row>
@@ -40869,54 +40861,54 @@
       <c r="C14" s="4" t="inlineStr"/>
       <c r="D14" s="4" t="inlineStr">
         <is>
+          <t>report_title</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Tên báo cáo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="4" t="inlineStr"/>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
           <t>prepared_by</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Đơn vị lập</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>manpower</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Nhan su theo thang</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Biểu đồ tăng cường nhân sự; KPI nhân sự lấy tháng cuối cùng có số thực tế</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Tháng, dạng YYYY-MM</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>onshore_plan</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Onshore kế hoạch</t>
         </is>
       </c>
     </row>
@@ -40926,12 +40918,12 @@
       <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>onshore_actual</t>
+          <t>onshore_plan</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Onshore thực tế (để trống nếu chưa tới)</t>
+          <t>Onshore kế hoạch</t>
         </is>
       </c>
     </row>
@@ -40941,12 +40933,12 @@
       <c r="C18" s="4" t="inlineStr"/>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>offshore_plan</t>
+          <t>onshore_actual</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Offshore kế hoạch</t>
+          <t>Onshore thực tế (để trống nếu chưa tới)</t>
         </is>
       </c>
     </row>
@@ -40956,12 +40948,12 @@
       <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>offshore_actual</t>
+          <t>offshore_plan</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Offshore thực tế</t>
+          <t>Offshore kế hoạch</t>
         </is>
       </c>
     </row>
@@ -40971,12 +40963,12 @@
       <c r="C20" s="4" t="inlineStr"/>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>total_plan</t>
+          <t>offshore_actual</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Tổng kế hoạch</t>
+          <t>Offshore thực tế</t>
         </is>
       </c>
     </row>
@@ -40986,54 +40978,54 @@
       <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="4" t="inlineStr">
         <is>
+          <t>total_plan</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Tổng kế hoạch</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr"/>
+      <c r="C22" s="4" t="inlineStr"/>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
           <t>total_actual</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>Tổng thực tế</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>staffing</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Dinh bien</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Thẻ "Định biên hiện tại"</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>group</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>Nhóm</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-      <c r="B23" s="4" t="inlineStr"/>
-      <c r="C23" s="4" t="inlineStr"/>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>filled</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Đã có</t>
         </is>
       </c>
     </row>
@@ -41043,54 +41035,54 @@
       <c r="C24" s="4" t="inlineStr"/>
       <c r="D24" s="4" t="inlineStr">
         <is>
+          <t>filled</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Đã có</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="4" t="inlineStr"/>
+      <c r="C25" s="4" t="inlineStr"/>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
           <t>required</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>Cần</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>cbta</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>CBTA</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Tab Nhân sự &amp; đào tạo: CBTA</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>platform</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>CPP hoặc WHP</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr"/>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>team</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Team</t>
         </is>
       </c>
     </row>
@@ -41100,12 +41092,12 @@
       <c r="C27" s="4" t="inlineStr"/>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>modules</t>
+          <t>team</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Tổng module</t>
+          <t>Team</t>
         </is>
       </c>
     </row>
@@ -41115,12 +41107,12 @@
       <c r="C28" s="4" t="inlineStr"/>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>developing</t>
+          <t>modules</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Đang biên soạn</t>
+          <t>Tổng module</t>
         </is>
       </c>
     </row>
@@ -41130,12 +41122,12 @@
       <c r="C29" s="4" t="inlineStr"/>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>developing</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Đang soát xét</t>
+          <t>Đang biên soạn</t>
         </is>
       </c>
     </row>
@@ -41145,12 +41137,12 @@
       <c r="C30" s="4" t="inlineStr"/>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>review</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Đã hoàn thành</t>
+          <t>Đang soát xét</t>
         </is>
       </c>
     </row>
@@ -41160,12 +41152,12 @@
       <c r="C31" s="4" t="inlineStr"/>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>theory_pct</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>% đánh giá lý thuyết (0–100)</t>
+          <t>Đã hoàn thành</t>
         </is>
       </c>
     </row>
@@ -41175,12 +41167,12 @@
       <c r="C32" s="4" t="inlineStr"/>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>ojt_modules</t>
+          <t>theory_pct</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Số module OJT</t>
+          <t>% đánh giá lý thuyết (0–100)</t>
         </is>
       </c>
     </row>
@@ -41190,54 +41182,54 @@
       <c r="C33" s="4" t="inlineStr"/>
       <c r="D33" s="4" t="inlineStr">
         <is>
+          <t>ojt_modules</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Số module OJT</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr"/>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
           <t>ojt_pct</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>% đánh giá OJT (0–100)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>mandatory</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Dao tao bat buoc</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Đào tạo bắt buộc offshore</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>team</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>Team</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr"/>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>planned</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Số khoá kế hoạch</t>
         </is>
       </c>
     </row>
@@ -41247,12 +41239,12 @@
       <c r="C36" s="4" t="inlineStr"/>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>earned</t>
+          <t>planned</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Số khoá đã hoàn thành</t>
+          <t>Số khoá kế hoạch</t>
         </is>
       </c>
     </row>
@@ -41262,96 +41254,96 @@
       <c r="C37" s="4" t="inlineStr"/>
       <c r="D37" s="4" t="inlineStr">
         <is>
+          <t>earned</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Số khoá đã hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr"/>
+      <c r="B38" s="4" t="inlineStr"/>
+      <c r="C38" s="4" t="inlineStr"/>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
           <t>balance</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>Còn lại</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>vendor_training</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Dao tao vendor</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Lịch đào tạo vendor</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>course</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>Tên khoá</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr"/>
-      <c r="B39" s="4" t="inlineStr"/>
-      <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr"/>
+      <c r="B40" s="4" t="inlineStr"/>
+      <c r="C40" s="4" t="inlineStr"/>
+      <c r="D40" s="4" t="inlineStr">
         <is>
           <t>period</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>Tháng YYYY-MM, hoặc chỉ năm YYYY</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>orr_teams</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>ORR theo team</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>ORR theo team OPS (tháng hiện tại)</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
         <is>
           <t>team</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>Team</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr"/>
-      <c r="B41" s="4" t="inlineStr"/>
-      <c r="C41" s="4" t="inlineStr"/>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>weight_pct</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>Trọng số %</t>
         </is>
       </c>
     </row>
@@ -41361,12 +41353,12 @@
       <c r="C42" s="4" t="inlineStr"/>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>total_activities</t>
+          <t>weight_pct</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Tổng hoạt động</t>
+          <t>Trọng số %</t>
         </is>
       </c>
     </row>
@@ -41376,12 +41368,12 @@
       <c r="C43" s="4" t="inlineStr"/>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>total_activities</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>Đã hoàn thành</t>
+          <t>Tổng hoạt động</t>
         </is>
       </c>
     </row>
@@ -41391,12 +41383,12 @@
       <c r="C44" s="4" t="inlineStr"/>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>plan_pct</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>% kế hoạch tháng hiện tại</t>
+          <t>Đã hoàn thành</t>
         </is>
       </c>
     </row>
@@ -41406,12 +41398,12 @@
       <c r="C45" s="4" t="inlineStr"/>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>actual_pct</t>
+          <t>plan_pct</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>% thực tế tháng hiện tại</t>
+          <t>% kế hoạch tháng hiện tại</t>
         </is>
       </c>
     </row>
@@ -41421,54 +41413,54 @@
       <c r="C46" s="4" t="inlineStr"/>
       <c r="D46" s="4" t="inlineStr">
         <is>
+          <t>actual_pct</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>% thực tế tháng hiện tại</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr"/>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
           <t>plan_end_pct</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>% kế hoạch cuối kỳ</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>orr_curve</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>ORR theo thang</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Đường ORR kế hoạch/thực tế; KPI ORR lấy tháng cuối cùng có thực tế</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>Tháng YYYY-MM</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr"/>
-      <c r="B48" s="4" t="inlineStr"/>
-      <c r="C48" s="4" t="inlineStr"/>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>plan_pct</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>% kế hoạch tổng</t>
         </is>
       </c>
     </row>
@@ -41478,54 +41470,54 @@
       <c r="C49" s="4" t="inlineStr"/>
       <c r="D49" s="4" t="inlineStr">
         <is>
+          <t>plan_pct</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>% kế hoạch tổng</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr"/>
+      <c r="B50" s="4" t="inlineStr"/>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
           <t>actual_pct</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="E50" s="4" t="inlineStr">
         <is>
           <t>% thực tế tổng (để trống nếu chưa tới)</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>orr_elements</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>ORR hang muc</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Bảng checklist theo hạng mục</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>group</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>PEOPLE / PLANT / PROCESS</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr"/>
-      <c r="B51" s="4" t="inlineStr"/>
-      <c r="C51" s="4" t="inlineStr"/>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>Mã (không trùng)</t>
         </is>
       </c>
     </row>
@@ -41535,12 +41527,12 @@
       <c r="C52" s="4" t="inlineStr"/>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>code</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Tên hạng mục</t>
+          <t>Mã (không trùng)</t>
         </is>
       </c>
     </row>
@@ -41550,12 +41542,12 @@
       <c r="C53" s="4" t="inlineStr"/>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>items</t>
+          <t>element</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Số đầu mục</t>
+          <t>Tên hạng mục</t>
         </is>
       </c>
     </row>
@@ -41565,54 +41557,54 @@
       <c r="C54" s="4" t="inlineStr"/>
       <c r="D54" s="4" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Số đầu mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr"/>
+      <c r="B55" s="4" t="inlineStr"/>
+      <c r="C55" s="4" t="inlineStr"/>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
           <t>progress_pct</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>% tiến độ (0–100)</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>orr_groups</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>ORR tong nhom</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Ô tổng ORR theo nhóm</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
         <is>
           <t>group</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>PEOPLE / PLANT / PROCESS / TOTAL (giữ nguyên tên)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr"/>
-      <c r="B56" s="4" t="inlineStr"/>
-      <c r="C56" s="4" t="inlineStr"/>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>items</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>Số đầu mục</t>
         </is>
       </c>
     </row>
@@ -41622,54 +41614,54 @@
       <c r="C57" s="4" t="inlineStr"/>
       <c r="D57" s="4" t="inlineStr">
         <is>
+          <t>items</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>Số đầu mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr"/>
+      <c r="B58" s="4" t="inlineStr"/>
+      <c r="C58" s="4" t="inlineStr"/>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
           <t>progress_pct</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>% tiến độ (0–100)</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>procedures</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>Quy trinh</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Tab Quy trình</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D59" s="4" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="E58" s="4" t="inlineStr">
+      <c r="E59" s="4" t="inlineStr">
         <is>
           <t>Mã (không trùng, ví dụ HSE-41)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr"/>
-      <c r="B59" s="4" t="inlineStr"/>
-      <c r="C59" s="4" t="inlineStr"/>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>"HSE" hoặc "General operations" (giữ đúng chữ)</t>
         </is>
       </c>
     </row>
@@ -41679,12 +41671,12 @@
       <c r="C60" s="4" t="inlineStr"/>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>document</t>
+          <t>category</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>Tên tài liệu</t>
+          <t>"HSE" hoặc "General operations" (giữ đúng chữ)</t>
         </is>
       </c>
     </row>
@@ -41694,12 +41686,12 @@
       <c r="C61" s="4" t="inlineStr"/>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>document</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>Company / Department</t>
+          <t>Tên tài liệu</t>
         </is>
       </c>
     </row>
@@ -41709,12 +41701,12 @@
       <c r="C62" s="4" t="inlineStr"/>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>issued</t>
+          <t>level</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>"Yes" nếu đã ban hành, "No" nếu chưa</t>
+          <t>Company / Department</t>
         </is>
       </c>
     </row>
@@ -41724,12 +41716,12 @@
       <c r="C63" s="4" t="inlineStr"/>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>responsible</t>
+          <t>issued</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>Người phụ trách</t>
+          <t>"Yes" nếu đã ban hành, "No" nếu chưa</t>
         </is>
       </c>
     </row>
@@ -41739,12 +41731,12 @@
       <c r="C64" s="4" t="inlineStr"/>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>expected</t>
+          <t>responsible</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>Hạn, ví dụ Dec-26</t>
+          <t>Người phụ trách</t>
         </is>
       </c>
     </row>
@@ -41754,12 +41746,12 @@
       <c r="C65" s="4" t="inlineStr"/>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>completion_pct</t>
+          <t>expected</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>% hoàn thành (0–100)</t>
+          <t>Hạn, ví dụ Dec-26</t>
         </is>
       </c>
     </row>
@@ -41769,54 +41761,54 @@
       <c r="C66" s="4" t="inlineStr"/>
       <c r="D66" s="4" t="inlineStr">
         <is>
+          <t>completion_pct</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>% hoàn thành (0–100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr"/>
+      <c r="B67" s="4" t="inlineStr"/>
+      <c r="C67" s="4" t="inlineStr"/>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
           <t>remark</t>
         </is>
       </c>
-      <c r="E66" s="4" t="inlineStr">
+      <c r="E67" s="4" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>packages_no_pr</t>
         </is>
       </c>
-      <c r="B67" s="4" t="inlineStr">
+      <c r="B68" s="4" t="inlineStr">
         <is>
           <t>Goi chua co PR</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>Gói chưa có PR</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="D68" s="4" t="inlineStr">
         <is>
           <t>dimension</t>
         </is>
       </c>
-      <c r="E67" s="4" t="inlineStr">
+      <c r="E68" s="4" t="inlineStr">
         <is>
           <t>status / priority / scr_timing (giữ nguyên)</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr"/>
-      <c r="B68" s="4" t="inlineStr"/>
-      <c r="C68" s="4" t="inlineStr"/>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>category</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>Nhóm</t>
         </is>
       </c>
     </row>
@@ -41826,54 +41818,54 @@
       <c r="C69" s="4" t="inlineStr"/>
       <c r="D69" s="4" t="inlineStr">
         <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>Nhóm</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr"/>
+      <c r="B70" s="4" t="inlineStr"/>
+      <c r="C70" s="4" t="inlineStr"/>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
           <t>count</t>
         </is>
       </c>
-      <c r="E69" s="4" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>Số gói</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>pr_pipeline</t>
         </is>
       </c>
-      <c r="B70" s="4" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>PR dang xu ly</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>PR theo bước</t>
         </is>
       </c>
-      <c r="D70" s="4" t="inlineStr">
+      <c r="D71" s="4" t="inlineStr">
         <is>
           <t>stage</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
+      <c r="E71" s="4" t="inlineStr">
         <is>
           <t>Bước (giữ số thứ tự ở đầu)</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr"/>
-      <c r="B71" s="4" t="inlineStr"/>
-      <c r="C71" s="4" t="inlineStr"/>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>"Late", "Near-late" hoặc "On time" (giữ đúng chữ)</t>
         </is>
       </c>
     </row>
@@ -41883,54 +41875,54 @@
       <c r="C72" s="4" t="inlineStr"/>
       <c r="D72" s="4" t="inlineStr">
         <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>"Late", "Near-late" hoặc "On time" (giữ đúng chữ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr"/>
+      <c r="B73" s="4" t="inlineStr"/>
+      <c r="C73" s="4" t="inlineStr"/>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
           <t>count</t>
         </is>
       </c>
-      <c r="E72" s="4" t="inlineStr">
+      <c r="E73" s="4" t="inlineStr">
         <is>
           <t>Số PR</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>cmms</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>CMMS</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>CMMS (OA)</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
+      <c r="D74" s="4" t="inlineStr">
         <is>
           <t>package</t>
         </is>
       </c>
-      <c r="E73" s="4" t="inlineStr">
+      <c r="E74" s="4" t="inlineStr">
         <is>
           <t>Gói</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="inlineStr"/>
-      <c r="B74" s="4" t="inlineStr"/>
-      <c r="C74" s="4" t="inlineStr"/>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>actual_pct</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>% thực tế</t>
         </is>
       </c>
     </row>
@@ -41940,54 +41932,54 @@
       <c r="C75" s="4" t="inlineStr"/>
       <c r="D75" s="4" t="inlineStr">
         <is>
+          <t>actual_pct</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>% thực tế</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr"/>
+      <c r="B76" s="4" t="inlineStr"/>
+      <c r="C76" s="4" t="inlineStr"/>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
           <t>plan_pct</t>
         </is>
       </c>
-      <c r="E75" s="4" t="inlineStr">
+      <c r="E76" s="4" t="inlineStr">
         <is>
           <t>% kế hoạch</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="4" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>workstreams</t>
         </is>
       </c>
-      <c r="B76" s="4" t="inlineStr">
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>Trang thai cong viec</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr">
+      <c r="C77" s="4" t="inlineStr">
         <is>
           <t>Danh sách ứng dụng, logistics, điều phối, commissioning, vị trí trống</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr">
+      <c r="D77" s="4" t="inlineStr">
         <is>
           <t>area</t>
         </is>
       </c>
-      <c r="E76" s="4" t="inlineStr">
+      <c r="E77" s="4" t="inlineStr">
         <is>
           <t>"Manpower", "Applications", "Logistics &amp; services", "Coordination" hoặc "Commissioning" (giữ đúng chữ)</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr"/>
-      <c r="B77" s="4" t="inlineStr"/>
-      <c r="C77" s="4" t="inlineStr"/>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>item</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>Hạng mục ("Vacant positions" là dòng vị trí còn trống)</t>
         </is>
       </c>
     </row>
@@ -41997,54 +41989,54 @@
       <c r="C78" s="4" t="inlineStr"/>
       <c r="D78" s="4" t="inlineStr">
         <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Hạng mục ("Vacant positions" là dòng vị trí còn trống)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr"/>
+      <c r="B79" s="4" t="inlineStr"/>
+      <c r="C79" s="4" t="inlineStr"/>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="E78" s="4" t="inlineStr">
+      <c r="E79" s="4" t="inlineStr">
         <is>
           <t>Trạng thái / bước tiếp theo</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>permits</t>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
+      <c r="B80" s="4" t="inlineStr">
         <is>
           <t>Giay phep</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>Đăng ký giấy phép</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr">
+      <c r="D80" s="4" t="inlineStr">
         <is>
           <t>permit</t>
         </is>
       </c>
-      <c r="E79" s="4" t="inlineStr">
+      <c r="E80" s="4" t="inlineStr">
         <is>
           <t>Tên giấy phép (không trùng)</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr"/>
-      <c r="B80" s="4" t="inlineStr"/>
-      <c r="C80" s="4" t="inlineStr"/>
-      <c r="D80" s="4" t="inlineStr">
-        <is>
-          <t>facility</t>
-        </is>
-      </c>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>Áp dụng cho</t>
         </is>
       </c>
     </row>
@@ -42054,12 +42046,12 @@
       <c r="C81" s="4" t="inlineStr"/>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>facility</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>Cơ quan</t>
+          <t>Áp dụng cho</t>
         </is>
       </c>
     </row>
@@ -42069,12 +42061,12 @@
       <c r="C82" s="4" t="inlineStr"/>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>issue_date</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>Ngày cấp YYYY-MM-DD</t>
+          <t>Cơ quan</t>
         </is>
       </c>
     </row>
@@ -42084,12 +42076,12 @@
       <c r="C83" s="4" t="inlineStr"/>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>expiry_date</t>
+          <t>issue_date</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>Ngày hết hạn YYYY-MM-DD</t>
+          <t>Ngày cấp YYYY-MM-DD</t>
         </is>
       </c>
     </row>
@@ -42099,12 +42091,12 @@
       <c r="C84" s="4" t="inlineStr"/>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>renewal_date</t>
+          <t>expiry_date</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Gia hạn trước YYYY-MM-DD</t>
+          <t>Ngày hết hạn YYYY-MM-DD</t>
         </is>
       </c>
     </row>
@@ -42114,54 +42106,54 @@
       <c r="C85" s="4" t="inlineStr"/>
       <c r="D85" s="4" t="inlineStr">
         <is>
+          <t>renewal_date</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Gia hạn trước YYYY-MM-DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr"/>
+      <c r="B86" s="4" t="inlineStr"/>
+      <c r="C86" s="4" t="inlineStr"/>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
           <t>status</t>
         </is>
       </c>
-      <c r="E85" s="4" t="inlineStr">
+      <c r="E86" s="4" t="inlineStr">
         <is>
           <t>"Issued", "Temporary", "Waiting…" hoặc ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="4" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
         <is>
           <t>precom_plan</t>
         </is>
       </c>
-      <c r="B86" s="4" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>Pre-com</t>
         </is>
       </c>
-      <c r="C86" s="4" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>Biểu đồ tiến độ pre-commissioning</t>
         </is>
       </c>
-      <c r="D86" s="4" t="inlineStr">
+      <c r="D87" s="4" t="inlineStr">
         <is>
           <t>activity</t>
         </is>
       </c>
-      <c r="E86" s="4" t="inlineStr">
+      <c r="E87" s="4" t="inlineStr">
         <is>
           <t>Tên hoạt động</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="4" t="inlineStr"/>
-      <c r="B87" s="4" t="inlineStr"/>
-      <c r="C87" s="4" t="inlineStr"/>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>plan_start</t>
-        </is>
-      </c>
-      <c r="E87" s="4" t="inlineStr">
-        <is>
-          <t>Bắt đầu KH YYYY-MM-DD</t>
         </is>
       </c>
     </row>
@@ -42171,12 +42163,12 @@
       <c r="C88" s="4" t="inlineStr"/>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>plan_finish</t>
+          <t>plan_start</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>Kết thúc KH YYYY-MM-DD</t>
+          <t>Bắt đầu KH YYYY-MM-DD</t>
         </is>
       </c>
     </row>
@@ -42186,12 +42178,12 @@
       <c r="C89" s="4" t="inlineStr"/>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>actual_start</t>
+          <t>plan_finish</t>
         </is>
       </c>
       <c r="E89" s="4" t="inlineStr">
         <is>
-          <t>Bắt đầu thực tế YYYY-MM-DD</t>
+          <t>Kết thúc KH YYYY-MM-DD</t>
         </is>
       </c>
     </row>
@@ -42201,54 +42193,54 @@
       <c r="C90" s="4" t="inlineStr"/>
       <c r="D90" s="4" t="inlineStr">
         <is>
+          <t>actual_start</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>Bắt đầu thực tế YYYY-MM-DD</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr"/>
+      <c r="B91" s="4" t="inlineStr"/>
+      <c r="C91" s="4" t="inlineStr"/>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
           <t>actual_finish</t>
         </is>
       </c>
-      <c r="E90" s="4" t="inlineStr">
+      <c r="E91" s="4" t="inlineStr">
         <is>
           <t>Kết thúc thực tế YYYY-MM-DD (có ngày → thanh màu xanh)</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="4" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
         <is>
           <t>startup_sequence</t>
         </is>
       </c>
-      <c r="B91" s="4" t="inlineStr">
+      <c r="B92" s="4" t="inlineStr">
         <is>
           <t>Trinh tu khoi dong</t>
         </is>
       </c>
-      <c r="C91" s="4" t="inlineStr">
+      <c r="C92" s="4" t="inlineStr">
         <is>
           <t>Trình tự khởi động CPP</t>
         </is>
       </c>
-      <c r="D91" s="4" t="inlineStr">
+      <c r="D92" s="4" t="inlineStr">
         <is>
           <t>step</t>
         </is>
       </c>
-      <c r="E91" s="4" t="inlineStr">
+      <c r="E92" s="4" t="inlineStr">
         <is>
           <t>Số thứ tự</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="4" t="inlineStr"/>
-      <c r="B92" s="4" t="inlineStr"/>
-      <c r="C92" s="4" t="inlineStr"/>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>phase</t>
-        </is>
-      </c>
-      <c r="E92" s="4" t="inlineStr">
-        <is>
-          <t>Tên bước</t>
         </is>
       </c>
     </row>
@@ -42258,10 +42250,25 @@
       <c r="C93" s="4" t="inlineStr"/>
       <c r="D93" s="4" t="inlineStr">
         <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>Tên bước</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr"/>
+      <c r="B94" s="4" t="inlineStr"/>
+      <c r="C94" s="4" t="inlineStr"/>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
           <t>action</t>
         </is>
       </c>
-      <c r="E93" s="4" t="inlineStr">
+      <c r="E94" s="4" t="inlineStr">
         <is>
           <t>Nội dung</t>
         </is>

</xml_diff>